<commit_message>
Upgrade de la lista de Materiales para compras, depósito y producción.
</commit_message>
<xml_diff>
--- a/Bill of Materials.xlsx
+++ b/Bill of Materials.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="86">
   <si>
     <t>Reference</t>
   </si>
@@ -265,6 +265,18 @@
   </si>
   <si>
     <t>Jumper_2_Open (1/4 de la tira por cada placa)</t>
+  </si>
+  <si>
+    <t>U0</t>
+  </si>
+  <si>
+    <t>Circuito Impreso ModemEYSE4G_LTE_Cat1_simcomA7670SA</t>
+  </si>
+  <si>
+    <t>W1</t>
+  </si>
+  <si>
+    <t>W2</t>
   </si>
 </sst>
 </file>
@@ -816,7 +828,7 @@
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -836,6 +848,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1163,7 +1178,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.140625" bestFit="1" customWidth="1"/>
@@ -1529,7 +1544,9 @@
       <c r="B22" s="3">
         <v>1</v>
       </c>
-      <c r="C22" s="3"/>
+      <c r="C22" s="3">
+        <v>60012938</v>
+      </c>
       <c r="D22" s="2" t="s">
         <v>37</v>
       </c>
@@ -1674,41 +1691,65 @@
       </c>
     </row>
     <row r="31" spans="1:5" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="2"/>
+      <c r="A31" s="2" t="s">
+        <v>82</v>
+      </c>
       <c r="B31" s="3">
         <v>1</v>
       </c>
       <c r="C31" s="3">
+        <v>10050108</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B32" s="3">
+        <v>1</v>
+      </c>
+      <c r="C32" s="3">
         <v>60004064</v>
       </c>
-      <c r="D31" s="2" t="s">
+      <c r="D32" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="E31" s="2" t="s">
+      <c r="E32" s="2" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="32" spans="1:5" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="2"/>
-      <c r="B32" s="3">
-        <v>1</v>
-      </c>
-      <c r="C32" s="3">
+    <row r="33" spans="1:5" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B33" s="3">
+        <v>1</v>
+      </c>
+      <c r="C33" s="3">
         <v>60004065</v>
       </c>
-      <c r="D32" s="2" t="s">
+      <c r="D33" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="E32" s="2" t="s">
+      <c r="E33" s="2" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="33" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="34" spans="1:5" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B35" s="9"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="53" fitToHeight="0" orientation="landscape" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="53" fitToHeight="0" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>